<commit_message>
Open invite links at top of page
</commit_message>
<xml_diff>
--- a/outputs/guest-list-template/sama-hisham-guest-list-links-ready.xlsx
+++ b/outputs/guest-list-template/sama-hisham-guest-list-links-ready.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sendable Links" sheetId="1" r:id="Rba8c05cf725e4500"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sendable Links" sheetId="1" r:id="R20dee4d2823a4f98"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -394,7 +394,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F2" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-7ba46443#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-7ba46443</x:v>
       </x:c>
       <x:c r="G2" s="6" t="str"/>
     </x:row>
@@ -415,7 +415,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F3" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-4889ac22#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-4889ac22</x:v>
       </x:c>
       <x:c r="G3" s="6" t="str"/>
     </x:row>
@@ -434,7 +434,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F4" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-805f1f1e#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-805f1f1e</x:v>
       </x:c>
       <x:c r="G4" s="6" t="str"/>
     </x:row>
@@ -453,7 +453,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F5" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-fc5acaae#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-fc5acaae</x:v>
       </x:c>
       <x:c r="G5" s="6" t="str"/>
     </x:row>
@@ -472,7 +472,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F6" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-c7607fc8#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-c7607fc8</x:v>
       </x:c>
       <x:c r="G6" s="6" t="str"/>
     </x:row>
@@ -491,7 +491,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F7" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-e40f156b#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-e40f156b</x:v>
       </x:c>
       <x:c r="G7" s="6" t="str"/>
     </x:row>
@@ -510,7 +510,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F8" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-c57bbd40#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-c57bbd40</x:v>
       </x:c>
       <x:c r="G8" s="6" t="str"/>
     </x:row>
@@ -529,7 +529,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F9" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-9082b25a#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-9082b25a</x:v>
       </x:c>
       <x:c r="G9" s="6" t="str"/>
     </x:row>
@@ -550,7 +550,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F10" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-69e47a8f#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-69e47a8f</x:v>
       </x:c>
       <x:c r="G10" s="6" t="str"/>
     </x:row>
@@ -571,7 +571,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F11" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-92abb076#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-92abb076</x:v>
       </x:c>
       <x:c r="G11" s="6" t="str"/>
     </x:row>
@@ -592,7 +592,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F12" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-a4b4ad54#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-a4b4ad54</x:v>
       </x:c>
       <x:c r="G12" s="6" t="str"/>
     </x:row>
@@ -611,7 +611,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F13" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-4fb2567d#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-4fb2567d</x:v>
       </x:c>
       <x:c r="G13" s="6" t="str"/>
     </x:row>
@@ -632,7 +632,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F14" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-6a7ad836#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-6a7ad836</x:v>
       </x:c>
       <x:c r="G14" s="6" t="str"/>
     </x:row>
@@ -651,7 +651,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F15" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-9ff70144#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-9ff70144</x:v>
       </x:c>
       <x:c r="G15" s="6" t="str"/>
     </x:row>
@@ -672,7 +672,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F16" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-d30fd0c4#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-d30fd0c4</x:v>
       </x:c>
       <x:c r="G16" s="6" t="str"/>
     </x:row>
@@ -691,7 +691,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F17" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-36c90253#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-36c90253</x:v>
       </x:c>
       <x:c r="G17" s="6" t="str"/>
     </x:row>
@@ -710,7 +710,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F18" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-f362ab7e#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-f362ab7e</x:v>
       </x:c>
       <x:c r="G18" s="6" t="str"/>
     </x:row>
@@ -731,7 +731,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F19" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-bcf90c3e#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-bcf90c3e</x:v>
       </x:c>
       <x:c r="G19" s="6" t="str"/>
     </x:row>
@@ -750,7 +750,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F20" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-027ca3e7#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-027ca3e7</x:v>
       </x:c>
       <x:c r="G20" s="6" t="str"/>
     </x:row>
@@ -769,7 +769,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F21" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-93924b80#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-93924b80</x:v>
       </x:c>
       <x:c r="G21" s="6" t="str"/>
     </x:row>
@@ -790,7 +790,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F22" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-e5ec3855#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-e5ec3855</x:v>
       </x:c>
       <x:c r="G22" s="6" t="str"/>
     </x:row>
@@ -809,7 +809,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F23" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-937630b4#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-937630b4</x:v>
       </x:c>
       <x:c r="G23" s="6" t="str"/>
     </x:row>
@@ -828,7 +828,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F24" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-999f3015#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-999f3015</x:v>
       </x:c>
       <x:c r="G24" s="6" t="str"/>
     </x:row>
@@ -847,7 +847,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F25" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-58206b68#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-58206b68</x:v>
       </x:c>
       <x:c r="G25" s="6" t="str"/>
     </x:row>
@@ -868,7 +868,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F26" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-ad99d16d#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-ad99d16d</x:v>
       </x:c>
       <x:c r="G26" s="6" t="str"/>
     </x:row>
@@ -887,7 +887,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F27" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-8cff1691#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-8cff1691</x:v>
       </x:c>
       <x:c r="G27" s="6" t="str"/>
     </x:row>
@@ -908,7 +908,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F28" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-dfdf3150#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-dfdf3150</x:v>
       </x:c>
       <x:c r="G28" s="6" t="str"/>
     </x:row>
@@ -927,7 +927,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F29" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-73f3c69d#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-73f3c69d</x:v>
       </x:c>
       <x:c r="G29" s="6" t="str"/>
     </x:row>
@@ -946,7 +946,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F30" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-3d86f9a7#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-3d86f9a7</x:v>
       </x:c>
       <x:c r="G30" s="6" t="str"/>
     </x:row>
@@ -965,7 +965,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F31" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-94c7fa2a#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-94c7fa2a</x:v>
       </x:c>
       <x:c r="G31" s="6" t="str"/>
     </x:row>
@@ -984,7 +984,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F32" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-aaff11f5#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-aaff11f5</x:v>
       </x:c>
       <x:c r="G32" s="6" t="str"/>
     </x:row>
@@ -1005,7 +1005,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F33" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-082ddbf9#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-082ddbf9</x:v>
       </x:c>
       <x:c r="G33" s="6" t="str"/>
     </x:row>
@@ -1024,7 +1024,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F34" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-6716c01a#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-6716c01a</x:v>
       </x:c>
       <x:c r="G34" s="6" t="str"/>
     </x:row>
@@ -1043,7 +1043,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F35" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-a745bb4f#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-a745bb4f</x:v>
       </x:c>
       <x:c r="G35" s="6" t="str"/>
     </x:row>
@@ -1064,7 +1064,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F36" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-18d0b1d8#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-18d0b1d8</x:v>
       </x:c>
       <x:c r="G36" s="6" t="str"/>
     </x:row>
@@ -1085,7 +1085,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F37" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-277ecb7f#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-277ecb7f</x:v>
       </x:c>
       <x:c r="G37" s="6" t="str"/>
     </x:row>
@@ -1106,7 +1106,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F38" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-057b9f69#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-057b9f69</x:v>
       </x:c>
       <x:c r="G38" s="6" t="str"/>
     </x:row>
@@ -1125,7 +1125,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F39" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-c71a4e38#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-c71a4e38</x:v>
       </x:c>
       <x:c r="G39" s="6" t="str"/>
     </x:row>
@@ -1144,7 +1144,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F40" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-93bc9347#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-93bc9347</x:v>
       </x:c>
       <x:c r="G40" s="6" t="str"/>
     </x:row>
@@ -1163,7 +1163,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F41" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-e26f9eed#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-e26f9eed</x:v>
       </x:c>
       <x:c r="G41" s="6" t="str"/>
     </x:row>
@@ -1182,7 +1182,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F42" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-35807d53#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-35807d53</x:v>
       </x:c>
       <x:c r="G42" s="6" t="str"/>
     </x:row>
@@ -1203,7 +1203,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F43" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-c13f3678#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-c13f3678</x:v>
       </x:c>
       <x:c r="G43" s="6" t="str"/>
     </x:row>
@@ -1222,7 +1222,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F44" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-a186c9d0#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-a186c9d0</x:v>
       </x:c>
       <x:c r="G44" s="6" t="str"/>
     </x:row>
@@ -1241,7 +1241,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F45" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-6e8c4ae6#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-6e8c4ae6</x:v>
       </x:c>
       <x:c r="G45" s="6" t="str"/>
     </x:row>
@@ -1262,7 +1262,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F46" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-4b8b739f#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-4b8b739f</x:v>
       </x:c>
       <x:c r="G46" s="6" t="str"/>
     </x:row>
@@ -1281,7 +1281,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F47" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-76093f64#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-76093f64</x:v>
       </x:c>
       <x:c r="G47" s="6" t="str"/>
     </x:row>
@@ -1300,7 +1300,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F48" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-ac02d588#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-ac02d588</x:v>
       </x:c>
       <x:c r="G48" s="6" t="str"/>
     </x:row>
@@ -1319,7 +1319,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F49" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-0fc06052#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-0fc06052</x:v>
       </x:c>
       <x:c r="G49" s="6" t="str"/>
     </x:row>
@@ -1338,7 +1338,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F50" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-e6210a51#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-e6210a51</x:v>
       </x:c>
       <x:c r="G50" s="6" t="str"/>
     </x:row>
@@ -1357,7 +1357,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F51" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-7ae4fb00#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-7ae4fb00</x:v>
       </x:c>
       <x:c r="G51" s="6" t="str"/>
     </x:row>
@@ -1376,7 +1376,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F52" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-f321ddf6#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-f321ddf6</x:v>
       </x:c>
       <x:c r="G52" s="6" t="str"/>
     </x:row>
@@ -1395,7 +1395,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F53" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-61ef57b1#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-61ef57b1</x:v>
       </x:c>
       <x:c r="G53" s="6" t="str"/>
     </x:row>
@@ -1416,7 +1416,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F54" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-834232bd#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-834232bd</x:v>
       </x:c>
       <x:c r="G54" s="6" t="str"/>
     </x:row>
@@ -1437,7 +1437,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F55" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-e39967ae#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-e39967ae</x:v>
       </x:c>
       <x:c r="G55" s="6" t="str"/>
     </x:row>
@@ -1456,7 +1456,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F56" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-22c9847a#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-22c9847a</x:v>
       </x:c>
       <x:c r="G56" s="6" t="str"/>
     </x:row>
@@ -1477,7 +1477,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F57" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-5a199723#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-5a199723</x:v>
       </x:c>
       <x:c r="G57" s="6" t="str"/>
     </x:row>
@@ -1496,7 +1496,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F58" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-9a5f330c#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-9a5f330c</x:v>
       </x:c>
       <x:c r="G58" s="6" t="str"/>
     </x:row>
@@ -1515,7 +1515,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F59" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-be101471#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-be101471</x:v>
       </x:c>
       <x:c r="G59" s="6" t="str"/>
     </x:row>
@@ -1534,7 +1534,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F60" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-591ba7f1#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-591ba7f1</x:v>
       </x:c>
       <x:c r="G60" s="6" t="str"/>
     </x:row>
@@ -1553,7 +1553,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F61" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-f8929a7d#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-f8929a7d</x:v>
       </x:c>
       <x:c r="G61" s="6" t="str"/>
     </x:row>
@@ -1572,7 +1572,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F62" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-13cbc4df#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-13cbc4df</x:v>
       </x:c>
       <x:c r="G62" s="6" t="str"/>
     </x:row>
@@ -1591,7 +1591,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F63" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-b70646d2#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-b70646d2</x:v>
       </x:c>
       <x:c r="G63" s="6" t="str"/>
     </x:row>
@@ -1610,7 +1610,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F64" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-2216dd54#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-2216dd54</x:v>
       </x:c>
       <x:c r="G64" s="6" t="str"/>
     </x:row>
@@ -1629,7 +1629,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F65" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-2e40bd22#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-2e40bd22</x:v>
       </x:c>
       <x:c r="G65" s="6" t="str"/>
     </x:row>
@@ -1648,7 +1648,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F66" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-8378d05c#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-8378d05c</x:v>
       </x:c>
       <x:c r="G66" s="6" t="str"/>
     </x:row>
@@ -1667,7 +1667,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F67" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-27b6526b#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-27b6526b</x:v>
       </x:c>
       <x:c r="G67" s="6" t="str"/>
     </x:row>
@@ -1686,7 +1686,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F68" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-baf50413#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-baf50413</x:v>
       </x:c>
       <x:c r="G68" s="6" t="str"/>
     </x:row>
@@ -1705,7 +1705,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F69" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-28b652b7#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-28b652b7</x:v>
       </x:c>
       <x:c r="G69" s="6" t="str"/>
     </x:row>
@@ -1724,7 +1724,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F70" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-8afaacfb#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-8afaacfb</x:v>
       </x:c>
       <x:c r="G70" s="6" t="str"/>
     </x:row>
@@ -1743,7 +1743,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F71" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-5406b30f#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-5406b30f</x:v>
       </x:c>
       <x:c r="G71" s="6" t="str"/>
     </x:row>
@@ -1762,7 +1762,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F72" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-0abb1097#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-0abb1097</x:v>
       </x:c>
       <x:c r="G72" s="6" t="str"/>
     </x:row>
@@ -1781,7 +1781,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F73" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-1d896892#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-1d896892</x:v>
       </x:c>
       <x:c r="G73" s="6" t="str"/>
     </x:row>
@@ -1800,7 +1800,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F74" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-36ac0fa6#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-36ac0fa6</x:v>
       </x:c>
       <x:c r="G74" s="6" t="str"/>
     </x:row>
@@ -1821,7 +1821,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F75" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-4378ce40#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-4378ce40</x:v>
       </x:c>
       <x:c r="G75" s="6" t="str"/>
     </x:row>
@@ -1840,7 +1840,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F76" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-10216ea4#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-10216ea4</x:v>
       </x:c>
       <x:c r="G76" s="6" t="str"/>
     </x:row>
@@ -1859,7 +1859,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F77" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-3ae74429#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-3ae74429</x:v>
       </x:c>
       <x:c r="G77" s="6" t="str"/>
     </x:row>
@@ -1878,7 +1878,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F78" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-242c483c#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-242c483c</x:v>
       </x:c>
       <x:c r="G78" s="6" t="str"/>
     </x:row>
@@ -1899,7 +1899,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F79" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-835955a9#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-835955a9</x:v>
       </x:c>
       <x:c r="G79" s="6" t="str"/>
     </x:row>
@@ -1920,7 +1920,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F80" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-dd63fa68#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-dd63fa68</x:v>
       </x:c>
       <x:c r="G80" s="6" t="str"/>
     </x:row>
@@ -1941,7 +1941,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F81" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-d23e9a42#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-d23e9a42</x:v>
       </x:c>
       <x:c r="G81" s="6" t="str"/>
     </x:row>
@@ -1962,7 +1962,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F82" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-b6327edc#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-b6327edc</x:v>
       </x:c>
       <x:c r="G82" s="6" t="str"/>
     </x:row>
@@ -1983,7 +1983,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F83" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-9b9d4ec4#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-9b9d4ec4</x:v>
       </x:c>
       <x:c r="G83" s="6" t="str"/>
     </x:row>
@@ -2002,7 +2002,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F84" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-276217af#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-276217af</x:v>
       </x:c>
       <x:c r="G84" s="6" t="str"/>
     </x:row>
@@ -2023,7 +2023,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F85" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-6680b4dd#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-6680b4dd</x:v>
       </x:c>
       <x:c r="G85" s="6" t="str"/>
     </x:row>
@@ -2042,7 +2042,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F86" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-06f081ea#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-06f081ea</x:v>
       </x:c>
       <x:c r="G86" s="6" t="str"/>
     </x:row>
@@ -2061,7 +2061,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F87" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-e859e31b#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-e859e31b</x:v>
       </x:c>
       <x:c r="G87" s="6" t="str"/>
     </x:row>
@@ -2080,7 +2080,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F88" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-0c130302#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-0c130302</x:v>
       </x:c>
       <x:c r="G88" s="6" t="str"/>
     </x:row>
@@ -2099,7 +2099,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F89" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-2102609e#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-2102609e</x:v>
       </x:c>
       <x:c r="G89" s="6" t="str"/>
     </x:row>
@@ -2118,7 +2118,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F90" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-b63d9a63#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-b63d9a63</x:v>
       </x:c>
       <x:c r="G90" s="6" t="str"/>
     </x:row>
@@ -2137,7 +2137,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F91" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-d686c9b1#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-d686c9b1</x:v>
       </x:c>
       <x:c r="G91" s="6" t="str"/>
     </x:row>
@@ -2156,7 +2156,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F92" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-45aadb19#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-45aadb19</x:v>
       </x:c>
       <x:c r="G92" s="6" t="str"/>
     </x:row>
@@ -2175,7 +2175,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F93" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-98c73a26#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-98c73a26</x:v>
       </x:c>
       <x:c r="G93" s="6" t="str"/>
     </x:row>
@@ -2194,7 +2194,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F94" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-3a8c995b#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-3a8c995b</x:v>
       </x:c>
       <x:c r="G94" s="6" t="str"/>
     </x:row>
@@ -2213,7 +2213,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F95" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-fdef4a10#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-fdef4a10</x:v>
       </x:c>
       <x:c r="G95" s="6" t="str"/>
     </x:row>
@@ -2232,7 +2232,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F96" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-d1dbab5b#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-d1dbab5b</x:v>
       </x:c>
       <x:c r="G96" s="6" t="str"/>
     </x:row>
@@ -2251,7 +2251,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F97" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-9719e2e5#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-9719e2e5</x:v>
       </x:c>
       <x:c r="G97" s="6" t="str"/>
     </x:row>
@@ -2270,7 +2270,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F98" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-d6631fdc#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-d6631fdc</x:v>
       </x:c>
       <x:c r="G98" s="6" t="str"/>
     </x:row>
@@ -2289,7 +2289,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F99" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-e354c183#rsvp</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-e354c183</x:v>
       </x:c>
       <x:c r="G99" s="6" t="str"/>
     </x:row>

</xml_diff>

<commit_message>
Add new RSVP guests
</commit_message>
<xml_diff>
--- a/outputs/guest-list-template/sama-hisham-guest-list-links-ready.xlsx
+++ b/outputs/guest-list-template/sama-hisham-guest-list-links-ready.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sendable Links" sheetId="1" r:id="R20dee4d2823a4f98"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sendable Links" sheetId="1" r:id="R4b664e7742474260"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2293,6 +2293,44 @@
       </x:c>
       <x:c r="G99" s="6" t="str"/>
     </x:row>
+    <x:row r="100">
+      <x:c r="A100" s="6" t="str">
+        <x:v>Mariam Hmedat</x:v>
+      </x:c>
+      <x:c r="B100" s="6" t="str">
+        <x:v>Mariam</x:v>
+      </x:c>
+      <x:c r="C100" s="20" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="D100" s="20" t="str"/>
+      <x:c r="E100" s="20" t="str">
+        <x:v>en</x:v>
+      </x:c>
+      <x:c r="F100" s="18" t="str">
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-14d80898</x:v>
+      </x:c>
+      <x:c r="G100" s="6" t="str"/>
+    </x:row>
+    <x:row r="101">
+      <x:c r="A101" s="6" t="str">
+        <x:v>Noura Afaneh</x:v>
+      </x:c>
+      <x:c r="B101" s="6" t="str">
+        <x:v>Noura</x:v>
+      </x:c>
+      <x:c r="C101" s="20" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="D101" s="20" t="str"/>
+      <x:c r="E101" s="20" t="str">
+        <x:v>en</x:v>
+      </x:c>
+      <x:c r="F101" s="18" t="str">
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-2d6295d4</x:v>
+      </x:c>
+      <x:c r="G101" s="6" t="str"/>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Add Yasmeen and Zeina invite links
</commit_message>
<xml_diff>
--- a/outputs/guest-list-template/sama-hisham-guest-list-links-ready.xlsx
+++ b/outputs/guest-list-template/sama-hisham-guest-list-links-ready.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sendable Links" sheetId="1" r:id="R4b664e7742474260"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sendable Links" sheetId="1" r:id="Rb35154e261c24d04"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2331,6 +2331,46 @@
       </x:c>
       <x:c r="G101" s="6" t="str"/>
     </x:row>
+    <x:row r="102">
+      <x:c r="A102" s="6" t="str">
+        <x:v>Yasmeen Hamad</x:v>
+      </x:c>
+      <x:c r="B102" s="6" t="str">
+        <x:v>Yasmeen</x:v>
+      </x:c>
+      <x:c r="C102" s="20" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="D102" s="20" t="str"/>
+      <x:c r="E102" s="20" t="str">
+        <x:v>en</x:v>
+      </x:c>
+      <x:c r="F102" s="18" t="str">
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-d33dc22e</x:v>
+      </x:c>
+      <x:c r="G102" s="6" t="str"/>
+    </x:row>
+    <x:row r="103">
+      <x:c r="A103" s="6" t="str">
+        <x:v>Zeina Barghouthi</x:v>
+      </x:c>
+      <x:c r="B103" s="6" t="str">
+        <x:v>Zeina</x:v>
+      </x:c>
+      <x:c r="C103" s="20" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="D103" s="20" t="str">
+        <x:v>Abed</x:v>
+      </x:c>
+      <x:c r="E103" s="20" t="str">
+        <x:v>en</x:v>
+      </x:c>
+      <x:c r="F103" s="18" t="str">
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-8355557e</x:v>
+      </x:c>
+      <x:c r="G103" s="6" t="str"/>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Add Rand and Aleen invite links
</commit_message>
<xml_diff>
--- a/outputs/guest-list-template/sama-hisham-guest-list-links-ready.xlsx
+++ b/outputs/guest-list-template/sama-hisham-guest-list-links-ready.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sendable Links" sheetId="1" r:id="Rb35154e261c24d04"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sendable Links" sheetId="1" r:id="R2cefa0c45fe846be"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2371,6 +2371,44 @@
       </x:c>
       <x:c r="G103" s="6" t="str"/>
     </x:row>
+    <x:row r="104">
+      <x:c r="A104" s="6" t="str">
+        <x:v>Rand Maslamani</x:v>
+      </x:c>
+      <x:c r="B104" s="6" t="str">
+        <x:v>Rand</x:v>
+      </x:c>
+      <x:c r="C104" s="20" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="D104" s="20" t="str"/>
+      <x:c r="E104" s="20" t="str">
+        <x:v>en</x:v>
+      </x:c>
+      <x:c r="F104" s="18" t="str">
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-a4fb7da5</x:v>
+      </x:c>
+      <x:c r="G104" s="6" t="str"/>
+    </x:row>
+    <x:row r="105">
+      <x:c r="A105" s="6" t="str">
+        <x:v>Aleen Shhab</x:v>
+      </x:c>
+      <x:c r="B105" s="6" t="str">
+        <x:v>Aleen</x:v>
+      </x:c>
+      <x:c r="C105" s="20" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="D105" s="20" t="str"/>
+      <x:c r="E105" s="20" t="str">
+        <x:v>en</x:v>
+      </x:c>
+      <x:c r="F105" s="18" t="str">
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-71b82287</x:v>
+      </x:c>
+      <x:c r="G105" s="6" t="str"/>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Add final RSVP links and extend deadline
</commit_message>
<xml_diff>
--- a/outputs/guest-list-template/sama-hisham-guest-list-links-ready.xlsx
+++ b/outputs/guest-list-template/sama-hisham-guest-list-links-ready.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sendable Links" sheetId="1" r:id="R2cefa0c45fe846be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sendable Links" sheetId="1" r:id="Race223c45d7d4dbc"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2200,10 +2200,10 @@
     </x:row>
     <x:row r="95">
       <x:c r="A95" s="6" t="str">
-        <x:v>Malak Dirawi</x:v>
+        <x:v>Cecilia Tannous</x:v>
       </x:c>
       <x:c r="B95" s="6" t="str">
-        <x:v>Malak</x:v>
+        <x:v>Cecilia</x:v>
       </x:c>
       <x:c r="C95" s="20" t="str">
         <x:v>no</x:v>
@@ -2408,6 +2408,120 @@
         <x:v>https://samaandhisham.vercel.app/?invite=sh-71b82287</x:v>
       </x:c>
       <x:c r="G105" s="6" t="str"/>
+    </x:row>
+    <x:row r="106">
+      <x:c r="A106" s="6" t="str">
+        <x:v>Hala Farraj</x:v>
+      </x:c>
+      <x:c r="B106" s="6" t="str">
+        <x:v>Hala</x:v>
+      </x:c>
+      <x:c r="C106" s="20" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="D106" s="20" t="str"/>
+      <x:c r="E106" s="20" t="str">
+        <x:v>en</x:v>
+      </x:c>
+      <x:c r="F106" s="18" t="str">
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-aa0a25ec</x:v>
+      </x:c>
+      <x:c r="G106" s="6" t="str"/>
+    </x:row>
+    <x:row r="107">
+      <x:c r="A107" s="6" t="str">
+        <x:v>Sari Jaber</x:v>
+      </x:c>
+      <x:c r="B107" s="6" t="str">
+        <x:v>Sari</x:v>
+      </x:c>
+      <x:c r="C107" s="20" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="D107" s="20" t="str"/>
+      <x:c r="E107" s="20" t="str">
+        <x:v>en</x:v>
+      </x:c>
+      <x:c r="F107" s="18" t="str">
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-43debabe</x:v>
+      </x:c>
+      <x:c r="G107" s="6" t="str"/>
+    </x:row>
+    <x:row r="108">
+      <x:c r="A108" s="6" t="str">
+        <x:v>Iman Irqat</x:v>
+      </x:c>
+      <x:c r="B108" s="6" t="str">
+        <x:v>Iman</x:v>
+      </x:c>
+      <x:c r="C108" s="20" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="D108" s="20" t="str"/>
+      <x:c r="E108" s="20" t="str">
+        <x:v>en</x:v>
+      </x:c>
+      <x:c r="F108" s="18" t="str">
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-d7ef039d</x:v>
+      </x:c>
+      <x:c r="G108" s="6" t="str"/>
+    </x:row>
+    <x:row r="109">
+      <x:c r="A109" s="6" t="str">
+        <x:v>Taleen Nasser</x:v>
+      </x:c>
+      <x:c r="B109" s="6" t="str">
+        <x:v>Taleen</x:v>
+      </x:c>
+      <x:c r="C109" s="20" t="str">
+        <x:v>no</x:v>
+      </x:c>
+      <x:c r="D109" s="20" t="str"/>
+      <x:c r="E109" s="20" t="str">
+        <x:v>en</x:v>
+      </x:c>
+      <x:c r="F109" s="18" t="str">
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-4ff54859</x:v>
+      </x:c>
+      <x:c r="G109" s="6" t="str"/>
+    </x:row>
+    <x:row r="110">
+      <x:c r="A110" s="6" t="str">
+        <x:v>Tamer Hinnawi</x:v>
+      </x:c>
+      <x:c r="B110" s="6" t="str">
+        <x:v>Tamer</x:v>
+      </x:c>
+      <x:c r="C110" s="20" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="D110" s="20" t="str"/>
+      <x:c r="E110" s="20" t="str">
+        <x:v>en</x:v>
+      </x:c>
+      <x:c r="F110" s="18" t="str">
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-db4db40c</x:v>
+      </x:c>
+      <x:c r="G110" s="6" t="str"/>
+    </x:row>
+    <x:row r="111">
+      <x:c r="A111" s="6" t="str">
+        <x:v>Awad Rimawi</x:v>
+      </x:c>
+      <x:c r="B111" s="6" t="str">
+        <x:v>Awad</x:v>
+      </x:c>
+      <x:c r="C111" s="20" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="D111" s="20" t="str"/>
+      <x:c r="E111" s="20" t="str">
+        <x:v>en</x:v>
+      </x:c>
+      <x:c r="F111" s="18" t="str">
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-72605248</x:v>
+      </x:c>
+      <x:c r="G111" s="6" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Update guest invite links
</commit_message>
<xml_diff>
--- a/outputs/guest-list-template/sama-hisham-guest-list-links-ready.xlsx
+++ b/outputs/guest-list-template/sama-hisham-guest-list-links-ready.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sendable Links" sheetId="1" r:id="Race223c45d7d4dbc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sendable Links" sheetId="1" r:id="Rff391f4567404a66"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -756,10 +756,10 @@
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="6" t="str">
-        <x:v>Hussam Omaia</x:v>
+        <x:v>Faleh Naseer Faleh</x:v>
       </x:c>
       <x:c r="B21" s="6" t="str">
-        <x:v>Hussam</x:v>
+        <x:v>Faleh</x:v>
       </x:c>
       <x:c r="C21" s="20" t="str">
         <x:v>no</x:v>
@@ -769,7 +769,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F21" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-93924b80</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-faleh-020</x:v>
       </x:c>
       <x:c r="G21" s="6" t="str"/>
     </x:row>
@@ -1559,10 +1559,10 @@
     </x:row>
     <x:row r="62">
       <x:c r="A62" s="6" t="str">
-        <x:v>Ziad rafidi</x:v>
+        <x:v>Dina Moghrabi</x:v>
       </x:c>
       <x:c r="B62" s="6" t="str">
-        <x:v>Ziad</x:v>
+        <x:v>Dina</x:v>
       </x:c>
       <x:c r="C62" s="20" t="str">
         <x:v>no</x:v>
@@ -1572,16 +1572,16 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F62" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-13cbc4df</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-dina-061</x:v>
       </x:c>
       <x:c r="G62" s="6" t="str"/>
     </x:row>
     <x:row r="63">
       <x:c r="A63" s="6" t="str">
-        <x:v>Majed Faraj</x:v>
+        <x:v>Areen Nassar</x:v>
       </x:c>
       <x:c r="B63" s="6" t="str">
-        <x:v>Majed</x:v>
+        <x:v>Areen</x:v>
       </x:c>
       <x:c r="C63" s="20" t="str">
         <x:v>yes</x:v>
@@ -1591,7 +1591,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F63" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-b70646d2</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-areen-062</x:v>
       </x:c>
       <x:c r="G63" s="6" t="str"/>
     </x:row>

</xml_diff>

<commit_message>
Update guest 41 invite link
</commit_message>
<xml_diff>
--- a/outputs/guest-list-template/sama-hisham-guest-list-links-ready.xlsx
+++ b/outputs/guest-list-template/sama-hisham-guest-list-links-ready.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sendable Links" sheetId="1" r:id="Rff391f4567404a66"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sendable Links" sheetId="1" r:id="Rf03b525279144d87"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1169,10 +1169,10 @@
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="6" t="str">
-        <x:v>Hasan Quweider</x:v>
+        <x:v>Amr marouf</x:v>
       </x:c>
       <x:c r="B42" s="6" t="str">
-        <x:v>Hassan</x:v>
+        <x:v>Amr</x:v>
       </x:c>
       <x:c r="C42" s="20" t="str">
         <x:v>no</x:v>
@@ -1182,7 +1182,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F42" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-35807d53</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-amr-041</x:v>
       </x:c>
       <x:c r="G42" s="6" t="str"/>
     </x:row>

</xml_diff>

<commit_message>
Update row 32 guest invite
</commit_message>
<xml_diff>
--- a/outputs/guest-list-template/sama-hisham-guest-list-links-ready.xlsx
+++ b/outputs/guest-list-template/sama-hisham-guest-list-links-ready.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sendable Links" sheetId="1" r:id="Rf03b525279144d87"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sendable Links" sheetId="1" r:id="R914a068dc0dd40ae"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -971,10 +971,10 @@
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="6" t="str">
-        <x:v>Yazan Abdulhadi</x:v>
+        <x:v>Saleem Malki</x:v>
       </x:c>
       <x:c r="B32" s="6" t="str">
-        <x:v>Yazan</x:v>
+        <x:v>Saleem</x:v>
       </x:c>
       <x:c r="C32" s="20" t="str">
         <x:v>yes</x:v>
@@ -984,7 +984,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="F32" s="18" t="str">
-        <x:v>https://samaandhisham.vercel.app/?invite=sh-aaff11f5</x:v>
+        <x:v>https://samaandhisham.vercel.app/?invite=sh-saleem-032</x:v>
       </x:c>
       <x:c r="G32" s="6" t="str"/>
     </x:row>

</xml_diff>